<commit_message>
Teensy blade control integration
</commit_message>
<xml_diff>
--- a/ArduinoCode/PGN OG3D.xlsx
+++ b/ArduinoCode/PGN OG3D.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="131">
   <si>
     <t xml:space="preserve">Format: 0x80, 0x81, Src, PGN, Length, [Data Bytes], CRC</t>
   </si>
@@ -221,145 +221,166 @@
     <t xml:space="preserve">E1</t>
   </si>
   <si>
+    <t xml:space="preserve">multipleStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwmValue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cutValve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BladeOffsetSlave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leverUpValue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">levelSideVal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwmHist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multiple bit:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0=up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1=down</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2=ready</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3=active</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data to valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int32 target altitude mm, &gt;20000 if none</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cut valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blade offset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">settings to valve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PwmGainUp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PwmGainDw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PwmMinUp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PwmMinDw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PwmMaxUp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PwmMaxDw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integal Multip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deadband</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Byte 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Byte 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Byte 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bautrate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">header hi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">header lo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB OG out  :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">relayRateData</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">option1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">option2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">option3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">option4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">relayRateSettings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">autoSteerData</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">autoSteerSettings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blade to OG3D (USB)</t>
+  </si>
+  <si>
     <t xml:space="preserve">valve direction</t>
   </si>
   <si>
-    <t xml:space="preserve">pwmValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cutValve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BladeOffsetSlave</t>
-  </si>
-  <si>
-    <t xml:space="preserve">leverUpValue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">levelSideVal</t>
+    <t xml:space="preserve">0 or 1</t>
   </si>
   <si>
     <t xml:space="preserve">bladeOffsetIn</t>
   </si>
   <si>
     <t xml:space="preserve">pwnHist</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data to valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">int32 target altitude mm, &gt;20000 if none</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cut valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blade offset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">settings to valve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PwmGainUp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PwmGainDw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PwmMinUp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PwmMinDw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PwmMaxUp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PwmMaxDw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integal Multip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deadband</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Byte 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Byte 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Byte 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bautrate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header hi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">header lo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB OG out  :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">relayRateData</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">option1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">option2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">option3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">option4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">relayRateSettings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">autoSteerData</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not used</t>
-  </si>
-  <si>
-    <t xml:space="preserve">autoSteerSettings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blade to OG3D (USB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 or 1</t>
   </si>
   <si>
     <t xml:space="preserve">IP Addresses when using fixed IPs</t>
@@ -2415,37 +2436,52 @@
       <c r="O7" s="4" t="s">
         <v>63</v>
       </c>
+      <c r="Q7" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>61</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>8</v>
       </c>
       <c r="G9" s="40" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H9" s="40"/>
       <c r="I9" s="40"/>
       <c r="J9" s="40"/>
       <c r="K9" s="4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L9" s="40" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="M9" s="40" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="O9" s="4" t="s">
         <v>63</v>
@@ -2465,40 +2501,40 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>61</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>8</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>63</v>
@@ -2532,13 +2568,13 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E16" s="17" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H16" s="18" t="s">
         <v>1</v>
@@ -2574,31 +2610,31 @@
         <v>16</v>
       </c>
       <c r="S16" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E17" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>127</v>
@@ -2607,22 +2643,22 @@
         <v>250</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2650,13 +2686,13 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>127</v>
@@ -2665,28 +2701,28 @@
         <v>248</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="S21" s="5" t="n">
         <v>38400</v>
@@ -2700,13 +2736,13 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>127</v>
@@ -2715,18 +2751,18 @@
         <v>254</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>127</v>
@@ -2735,18 +2771,18 @@
         <v>252</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" s="47" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="42" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B26" s="43"/>
       <c r="C26" s="43"/>
       <c r="D26" s="43"/>
       <c r="E26" s="43" t="s">
-        <v>66</v>
+        <v>116</v>
       </c>
       <c r="F26" s="44" t="s">
         <v>67</v>
@@ -2758,16 +2794,16 @@
         <v>69</v>
       </c>
       <c r="I26" s="45" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J26" s="45" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="K26" s="45" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L26" s="45" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="M26" s="45"/>
       <c r="N26" s="45"/>
@@ -2783,7 +2819,7 @@
       <c r="C27" s="7"/>
       <c r="D27" s="7"/>
       <c r="E27" s="7" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="40"/>
@@ -2795,10 +2831,10 @@
         <v>71</v>
       </c>
       <c r="K27" s="40" t="s">
-        <v>72</v>
+        <v>118</v>
       </c>
       <c r="L27" s="40" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="M27" s="40"/>
       <c r="N27" s="40"/>
@@ -2908,17 +2944,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="54" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="55" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="53" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2926,7 +2962,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="53" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2934,10 +2970,10 @@
         <v>71</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C7" s="53" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2945,10 +2981,10 @@
         <v>72</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C8" s="53" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2966,10 +3002,10 @@
         <v>75</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C11" s="53" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2977,10 +3013,10 @@
         <v>76</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C12" s="53" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2988,10 +3024,10 @@
         <v>77</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C13" s="53" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2999,10 +3035,10 @@
         <v>78</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C14" s="53" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3010,10 +3046,10 @@
         <v>79</v>
       </c>
       <c r="B15" s="53" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C15" s="53" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3021,10 +3057,10 @@
         <v>80</v>
       </c>
       <c r="B16" s="53" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="C16" s="53" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3042,7 +3078,7 @@
         <v>100</v>
       </c>
       <c r="B22" s="53" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>